<commit_message>
release: RC Go/No-Go (NO-GO today), merge checklist, Supabase readiness; incident narrowed; R&D units KG/EA/Pack/Carton
- Firestore 4-9 Oct hourly metrics (owner project): ~630K reads in bursts 6 Oct 20:00 -> 7 Oct
  10:00 ICT while rule evaluations stayed normal: the excess bypassed the rules (admin/service
  account/console), not the app's users. Incident stays OPEN, narrowed.
- Previews now behind Cloudflare Access (*.pzmstock.pages.dev); production unaffected (re-probed).
- R&D unit template: only the other brands' units with Carton instead of Bottle; suggestions
  only where the same product exists in Pizza Mania / Le Lapin (17 of 228), never applied.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ops/rnd-units-template.xlsx
+++ b/docs/ops/rnd-units-template.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I229"/>
+  <dimension ref="A1:K229"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -417,15 +417,21 @@
         <v>currentUnit</v>
       </c>
       <c r="F1" t="str">
+        <v>suggestedUnit</v>
+      </c>
+      <c r="G1" t="str">
+        <v>suggestedFrom</v>
+      </c>
+      <c r="H1" t="str">
         <v>proposedUnit</v>
       </c>
-      <c r="G1" t="str">
+      <c r="I1" t="str">
         <v>baseUnit</v>
       </c>
-      <c r="H1" t="str">
+      <c r="J1" t="str">
         <v>conversionFactor</v>
       </c>
-      <c r="I1" t="str">
+      <c r="K1" t="str">
         <v>validationStatus</v>
       </c>
     </row>
@@ -455,6 +461,12 @@
         <v/>
       </c>
       <c r="I2" t="str">
+        <v/>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -484,6 +496,12 @@
         <v/>
       </c>
       <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -513,6 +531,12 @@
         <v/>
       </c>
       <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
+      <c r="K4" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -542,6 +566,12 @@
         <v/>
       </c>
       <c r="I5" t="str">
+        <v/>
+      </c>
+      <c r="J5" t="str">
+        <v/>
+      </c>
+      <c r="K5" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -571,6 +601,12 @@
         <v/>
       </c>
       <c r="I6" t="str">
+        <v/>
+      </c>
+      <c r="J6" t="str">
+        <v/>
+      </c>
+      <c r="K6" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -600,6 +636,12 @@
         <v/>
       </c>
       <c r="I7" t="str">
+        <v/>
+      </c>
+      <c r="J7" t="str">
+        <v/>
+      </c>
+      <c r="K7" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -629,6 +671,12 @@
         <v/>
       </c>
       <c r="I8" t="str">
+        <v/>
+      </c>
+      <c r="J8" t="str">
+        <v/>
+      </c>
+      <c r="K8" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -658,6 +706,12 @@
         <v/>
       </c>
       <c r="I9" t="str">
+        <v/>
+      </c>
+      <c r="J9" t="str">
+        <v/>
+      </c>
+      <c r="K9" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -687,6 +741,12 @@
         <v/>
       </c>
       <c r="I10" t="str">
+        <v/>
+      </c>
+      <c r="J10" t="str">
+        <v/>
+      </c>
+      <c r="K10" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -716,6 +776,12 @@
         <v/>
       </c>
       <c r="I11" t="str">
+        <v/>
+      </c>
+      <c r="J11" t="str">
+        <v/>
+      </c>
+      <c r="K11" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -745,6 +811,12 @@
         <v/>
       </c>
       <c r="I12" t="str">
+        <v/>
+      </c>
+      <c r="J12" t="str">
+        <v/>
+      </c>
+      <c r="K12" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -774,6 +846,12 @@
         <v/>
       </c>
       <c r="I13" t="str">
+        <v/>
+      </c>
+      <c r="J13" t="str">
+        <v/>
+      </c>
+      <c r="K13" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -803,6 +881,12 @@
         <v/>
       </c>
       <c r="I14" t="str">
+        <v/>
+      </c>
+      <c r="J14" t="str">
+        <v/>
+      </c>
+      <c r="K14" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -832,6 +916,12 @@
         <v/>
       </c>
       <c r="I15" t="str">
+        <v/>
+      </c>
+      <c r="J15" t="str">
+        <v/>
+      </c>
+      <c r="K15" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -861,6 +951,12 @@
         <v/>
       </c>
       <c r="I16" t="str">
+        <v/>
+      </c>
+      <c r="J16" t="str">
+        <v/>
+      </c>
+      <c r="K16" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -890,6 +986,12 @@
         <v/>
       </c>
       <c r="I17" t="str">
+        <v/>
+      </c>
+      <c r="J17" t="str">
+        <v/>
+      </c>
+      <c r="K17" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -910,15 +1012,21 @@
         <v/>
       </c>
       <c r="F18" t="str">
-        <v/>
+        <v>KG</v>
       </c>
       <c r="G18" t="str">
-        <v/>
+        <v>Pizza Mania VGT-01-11-004; Pizza Mania VGT-01-11-005; Le Lapin VGT-LL-01-21-001</v>
       </c>
       <c r="H18" t="str">
         <v/>
       </c>
       <c r="I18" t="str">
+        <v/>
+      </c>
+      <c r="J18" t="str">
+        <v/>
+      </c>
+      <c r="K18" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -939,15 +1047,21 @@
         <v/>
       </c>
       <c r="F19" t="str">
-        <v/>
+        <v>KG</v>
       </c>
       <c r="G19" t="str">
-        <v/>
+        <v>Pizza Mania VGT-01-11-004; Pizza Mania VGT-01-11-005; Le Lapin VGT-LL-01-21-001</v>
       </c>
       <c r="H19" t="str">
         <v/>
       </c>
       <c r="I19" t="str">
+        <v/>
+      </c>
+      <c r="J19" t="str">
+        <v/>
+      </c>
+      <c r="K19" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -977,6 +1091,12 @@
         <v/>
       </c>
       <c r="I20" t="str">
+        <v/>
+      </c>
+      <c r="J20" t="str">
+        <v/>
+      </c>
+      <c r="K20" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1006,6 +1126,12 @@
         <v/>
       </c>
       <c r="I21" t="str">
+        <v/>
+      </c>
+      <c r="J21" t="str">
+        <v/>
+      </c>
+      <c r="K21" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1026,15 +1152,21 @@
         <v/>
       </c>
       <c r="F22" t="str">
-        <v/>
+        <v>KG</v>
       </c>
       <c r="G22" t="str">
-        <v/>
+        <v>Le Lapin VGT-LL-01-13-003; Le Lapin VGT-LL-01-13-004</v>
       </c>
       <c r="H22" t="str">
         <v/>
       </c>
       <c r="I22" t="str">
+        <v/>
+      </c>
+      <c r="J22" t="str">
+        <v/>
+      </c>
+      <c r="K22" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1055,15 +1187,21 @@
         <v/>
       </c>
       <c r="F23" t="str">
-        <v/>
+        <v>KG</v>
       </c>
       <c r="G23" t="str">
-        <v/>
+        <v>Le Lapin VGT-LL-01-13-003; Le Lapin VGT-LL-01-13-004</v>
       </c>
       <c r="H23" t="str">
         <v/>
       </c>
       <c r="I23" t="str">
+        <v/>
+      </c>
+      <c r="J23" t="str">
+        <v/>
+      </c>
+      <c r="K23" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1093,6 +1231,12 @@
         <v/>
       </c>
       <c r="I24" t="str">
+        <v/>
+      </c>
+      <c r="J24" t="str">
+        <v/>
+      </c>
+      <c r="K24" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1113,15 +1257,21 @@
         <v/>
       </c>
       <c r="F25" t="str">
-        <v/>
+        <v>KG</v>
       </c>
       <c r="G25" t="str">
-        <v/>
+        <v>Le Lapin VGT-LL-01-10-002; Le Lapin VGT-LL-01-10-003</v>
       </c>
       <c r="H25" t="str">
         <v/>
       </c>
       <c r="I25" t="str">
+        <v/>
+      </c>
+      <c r="J25" t="str">
+        <v/>
+      </c>
+      <c r="K25" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1142,15 +1292,21 @@
         <v/>
       </c>
       <c r="F26" t="str">
-        <v/>
+        <v>KG</v>
       </c>
       <c r="G26" t="str">
-        <v/>
+        <v>Le Lapin VGT-LL-01-10-002; Le Lapin VGT-LL-01-10-003</v>
       </c>
       <c r="H26" t="str">
         <v/>
       </c>
       <c r="I26" t="str">
+        <v/>
+      </c>
+      <c r="J26" t="str">
+        <v/>
+      </c>
+      <c r="K26" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1180,6 +1336,12 @@
         <v/>
       </c>
       <c r="I27" t="str">
+        <v/>
+      </c>
+      <c r="J27" t="str">
+        <v/>
+      </c>
+      <c r="K27" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1209,6 +1371,12 @@
         <v/>
       </c>
       <c r="I28" t="str">
+        <v/>
+      </c>
+      <c r="J28" t="str">
+        <v/>
+      </c>
+      <c r="K28" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1238,6 +1406,12 @@
         <v/>
       </c>
       <c r="I29" t="str">
+        <v/>
+      </c>
+      <c r="J29" t="str">
+        <v/>
+      </c>
+      <c r="K29" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1267,6 +1441,12 @@
         <v/>
       </c>
       <c r="I30" t="str">
+        <v/>
+      </c>
+      <c r="J30" t="str">
+        <v/>
+      </c>
+      <c r="K30" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1296,6 +1476,12 @@
         <v/>
       </c>
       <c r="I31" t="str">
+        <v/>
+      </c>
+      <c r="J31" t="str">
+        <v/>
+      </c>
+      <c r="K31" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1325,6 +1511,12 @@
         <v/>
       </c>
       <c r="I32" t="str">
+        <v/>
+      </c>
+      <c r="J32" t="str">
+        <v/>
+      </c>
+      <c r="K32" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1354,6 +1546,12 @@
         <v/>
       </c>
       <c r="I33" t="str">
+        <v/>
+      </c>
+      <c r="J33" t="str">
+        <v/>
+      </c>
+      <c r="K33" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1383,6 +1581,12 @@
         <v/>
       </c>
       <c r="I34" t="str">
+        <v/>
+      </c>
+      <c r="J34" t="str">
+        <v/>
+      </c>
+      <c r="K34" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1412,6 +1616,12 @@
         <v/>
       </c>
       <c r="I35" t="str">
+        <v/>
+      </c>
+      <c r="J35" t="str">
+        <v/>
+      </c>
+      <c r="K35" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1441,6 +1651,12 @@
         <v/>
       </c>
       <c r="I36" t="str">
+        <v/>
+      </c>
+      <c r="J36" t="str">
+        <v/>
+      </c>
+      <c r="K36" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1461,15 +1677,21 @@
         <v/>
       </c>
       <c r="F37" t="str">
-        <v/>
+        <v>KG</v>
       </c>
       <c r="G37" t="str">
-        <v/>
+        <v>Pizza Mania VGT-01-13-002; Pizza Mania VGT-01-13-003; Pizza Mania VGT-01-13-004; Le Lapin VGT-LL-01-12-001; Le Lapin VGT-LL-01-12-002; Le Lapin VGT-LL-01-12-003; Le Lapin VGT-LL-01-12-004</v>
       </c>
       <c r="H37" t="str">
         <v/>
       </c>
       <c r="I37" t="str">
+        <v/>
+      </c>
+      <c r="J37" t="str">
+        <v/>
+      </c>
+      <c r="K37" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1499,6 +1721,12 @@
         <v/>
       </c>
       <c r="I38" t="str">
+        <v/>
+      </c>
+      <c r="J38" t="str">
+        <v/>
+      </c>
+      <c r="K38" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1528,6 +1756,12 @@
         <v/>
       </c>
       <c r="I39" t="str">
+        <v/>
+      </c>
+      <c r="J39" t="str">
+        <v/>
+      </c>
+      <c r="K39" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1548,15 +1782,21 @@
         <v/>
       </c>
       <c r="F40" t="str">
-        <v/>
+        <v>KG</v>
       </c>
       <c r="G40" t="str">
-        <v/>
+        <v>Pizza Mania VGT-01-05-003; Pizza Mania VGT-01-05-004; Pizza Mania VGT-01-05-005; Pizza Mania VGT-01-05-006; Le Lapin VGT-LL-01-18-001</v>
       </c>
       <c r="H40" t="str">
         <v/>
       </c>
       <c r="I40" t="str">
+        <v/>
+      </c>
+      <c r="J40" t="str">
+        <v/>
+      </c>
+      <c r="K40" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1586,6 +1826,12 @@
         <v/>
       </c>
       <c r="I41" t="str">
+        <v/>
+      </c>
+      <c r="J41" t="str">
+        <v/>
+      </c>
+      <c r="K41" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1606,15 +1852,21 @@
         <v/>
       </c>
       <c r="F42" t="str">
-        <v/>
+        <v>KG</v>
       </c>
       <c r="G42" t="str">
-        <v/>
+        <v>Pizza Mania VGT-01-18-002</v>
       </c>
       <c r="H42" t="str">
         <v/>
       </c>
       <c r="I42" t="str">
+        <v/>
+      </c>
+      <c r="J42" t="str">
+        <v/>
+      </c>
+      <c r="K42" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1635,15 +1887,21 @@
         <v/>
       </c>
       <c r="F43" t="str">
-        <v/>
+        <v>KG</v>
       </c>
       <c r="G43" t="str">
-        <v/>
+        <v>Pizza Mania VGT-01-02-014; Pizza Mania VGT-01-02-017</v>
       </c>
       <c r="H43" t="str">
         <v/>
       </c>
       <c r="I43" t="str">
+        <v/>
+      </c>
+      <c r="J43" t="str">
+        <v/>
+      </c>
+      <c r="K43" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1664,15 +1922,21 @@
         <v/>
       </c>
       <c r="F44" t="str">
-        <v/>
+        <v>KG</v>
       </c>
       <c r="G44" t="str">
-        <v/>
+        <v>Pizza Mania VGT-01-02-015; Pizza Mania VGT-01-02-018</v>
       </c>
       <c r="H44" t="str">
         <v/>
       </c>
       <c r="I44" t="str">
+        <v/>
+      </c>
+      <c r="J44" t="str">
+        <v/>
+      </c>
+      <c r="K44" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1693,15 +1957,21 @@
         <v/>
       </c>
       <c r="F45" t="str">
-        <v/>
+        <v>KG</v>
       </c>
       <c r="G45" t="str">
-        <v/>
+        <v>Pizza Mania VGT-01-02-016; Pizza Mania VGT-01-02-019</v>
       </c>
       <c r="H45" t="str">
         <v/>
       </c>
       <c r="I45" t="str">
+        <v/>
+      </c>
+      <c r="J45" t="str">
+        <v/>
+      </c>
+      <c r="K45" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1731,6 +2001,12 @@
         <v/>
       </c>
       <c r="I46" t="str">
+        <v/>
+      </c>
+      <c r="J46" t="str">
+        <v/>
+      </c>
+      <c r="K46" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1760,6 +2036,12 @@
         <v/>
       </c>
       <c r="I47" t="str">
+        <v/>
+      </c>
+      <c r="J47" t="str">
+        <v/>
+      </c>
+      <c r="K47" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1789,6 +2071,12 @@
         <v/>
       </c>
       <c r="I48" t="str">
+        <v/>
+      </c>
+      <c r="J48" t="str">
+        <v/>
+      </c>
+      <c r="K48" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1818,6 +2106,12 @@
         <v/>
       </c>
       <c r="I49" t="str">
+        <v/>
+      </c>
+      <c r="J49" t="str">
+        <v/>
+      </c>
+      <c r="K49" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1847,6 +2141,12 @@
         <v/>
       </c>
       <c r="I50" t="str">
+        <v/>
+      </c>
+      <c r="J50" t="str">
+        <v/>
+      </c>
+      <c r="K50" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1876,6 +2176,12 @@
         <v/>
       </c>
       <c r="I51" t="str">
+        <v/>
+      </c>
+      <c r="J51" t="str">
+        <v/>
+      </c>
+      <c r="K51" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1905,6 +2211,12 @@
         <v/>
       </c>
       <c r="I52" t="str">
+        <v/>
+      </c>
+      <c r="J52" t="str">
+        <v/>
+      </c>
+      <c r="K52" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1934,6 +2246,12 @@
         <v/>
       </c>
       <c r="I53" t="str">
+        <v/>
+      </c>
+      <c r="J53" t="str">
+        <v/>
+      </c>
+      <c r="K53" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1963,6 +2281,12 @@
         <v/>
       </c>
       <c r="I54" t="str">
+        <v/>
+      </c>
+      <c r="J54" t="str">
+        <v/>
+      </c>
+      <c r="K54" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -1992,6 +2316,12 @@
         <v/>
       </c>
       <c r="I55" t="str">
+        <v/>
+      </c>
+      <c r="J55" t="str">
+        <v/>
+      </c>
+      <c r="K55" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2021,6 +2351,12 @@
         <v/>
       </c>
       <c r="I56" t="str">
+        <v/>
+      </c>
+      <c r="J56" t="str">
+        <v/>
+      </c>
+      <c r="K56" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2050,6 +2386,12 @@
         <v/>
       </c>
       <c r="I57" t="str">
+        <v/>
+      </c>
+      <c r="J57" t="str">
+        <v/>
+      </c>
+      <c r="K57" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2079,6 +2421,12 @@
         <v/>
       </c>
       <c r="I58" t="str">
+        <v/>
+      </c>
+      <c r="J58" t="str">
+        <v/>
+      </c>
+      <c r="K58" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2108,6 +2456,12 @@
         <v/>
       </c>
       <c r="I59" t="str">
+        <v/>
+      </c>
+      <c r="J59" t="str">
+        <v/>
+      </c>
+      <c r="K59" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2137,6 +2491,12 @@
         <v/>
       </c>
       <c r="I60" t="str">
+        <v/>
+      </c>
+      <c r="J60" t="str">
+        <v/>
+      </c>
+      <c r="K60" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2166,6 +2526,12 @@
         <v/>
       </c>
       <c r="I61" t="str">
+        <v/>
+      </c>
+      <c r="J61" t="str">
+        <v/>
+      </c>
+      <c r="K61" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2195,6 +2561,12 @@
         <v/>
       </c>
       <c r="I62" t="str">
+        <v/>
+      </c>
+      <c r="J62" t="str">
+        <v/>
+      </c>
+      <c r="K62" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2224,6 +2596,12 @@
         <v/>
       </c>
       <c r="I63" t="str">
+        <v/>
+      </c>
+      <c r="J63" t="str">
+        <v/>
+      </c>
+      <c r="K63" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2253,6 +2631,12 @@
         <v/>
       </c>
       <c r="I64" t="str">
+        <v/>
+      </c>
+      <c r="J64" t="str">
+        <v/>
+      </c>
+      <c r="K64" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2282,6 +2666,12 @@
         <v/>
       </c>
       <c r="I65" t="str">
+        <v/>
+      </c>
+      <c r="J65" t="str">
+        <v/>
+      </c>
+      <c r="K65" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2311,6 +2701,12 @@
         <v/>
       </c>
       <c r="I66" t="str">
+        <v/>
+      </c>
+      <c r="J66" t="str">
+        <v/>
+      </c>
+      <c r="K66" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2340,6 +2736,12 @@
         <v/>
       </c>
       <c r="I67" t="str">
+        <v/>
+      </c>
+      <c r="J67" t="str">
+        <v/>
+      </c>
+      <c r="K67" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2369,6 +2771,12 @@
         <v/>
       </c>
       <c r="I68" t="str">
+        <v/>
+      </c>
+      <c r="J68" t="str">
+        <v/>
+      </c>
+      <c r="K68" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2398,6 +2806,12 @@
         <v/>
       </c>
       <c r="I69" t="str">
+        <v/>
+      </c>
+      <c r="J69" t="str">
+        <v/>
+      </c>
+      <c r="K69" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2427,6 +2841,12 @@
         <v/>
       </c>
       <c r="I70" t="str">
+        <v/>
+      </c>
+      <c r="J70" t="str">
+        <v/>
+      </c>
+      <c r="K70" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2456,6 +2876,12 @@
         <v/>
       </c>
       <c r="I71" t="str">
+        <v/>
+      </c>
+      <c r="J71" t="str">
+        <v/>
+      </c>
+      <c r="K71" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2485,6 +2911,12 @@
         <v/>
       </c>
       <c r="I72" t="str">
+        <v/>
+      </c>
+      <c r="J72" t="str">
+        <v/>
+      </c>
+      <c r="K72" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2514,6 +2946,12 @@
         <v/>
       </c>
       <c r="I73" t="str">
+        <v/>
+      </c>
+      <c r="J73" t="str">
+        <v/>
+      </c>
+      <c r="K73" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2543,6 +2981,12 @@
         <v/>
       </c>
       <c r="I74" t="str">
+        <v/>
+      </c>
+      <c r="J74" t="str">
+        <v/>
+      </c>
+      <c r="K74" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2572,6 +3016,12 @@
         <v/>
       </c>
       <c r="I75" t="str">
+        <v/>
+      </c>
+      <c r="J75" t="str">
+        <v/>
+      </c>
+      <c r="K75" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2592,15 +3042,21 @@
         <v/>
       </c>
       <c r="F76" t="str">
-        <v/>
+        <v>KG</v>
       </c>
       <c r="G76" t="str">
-        <v/>
+        <v>Pizza Mania MES-01-15-007</v>
       </c>
       <c r="H76" t="str">
         <v/>
       </c>
       <c r="I76" t="str">
+        <v/>
+      </c>
+      <c r="J76" t="str">
+        <v/>
+      </c>
+      <c r="K76" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2621,15 +3077,21 @@
         <v/>
       </c>
       <c r="F77" t="str">
-        <v/>
+        <v>KG</v>
       </c>
       <c r="G77" t="str">
-        <v/>
+        <v>Pizza Mania MES-01-15-008</v>
       </c>
       <c r="H77" t="str">
         <v/>
       </c>
       <c r="I77" t="str">
+        <v/>
+      </c>
+      <c r="J77" t="str">
+        <v/>
+      </c>
+      <c r="K77" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2659,6 +3121,12 @@
         <v/>
       </c>
       <c r="I78" t="str">
+        <v/>
+      </c>
+      <c r="J78" t="str">
+        <v/>
+      </c>
+      <c r="K78" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2688,6 +3156,12 @@
         <v/>
       </c>
       <c r="I79" t="str">
+        <v/>
+      </c>
+      <c r="J79" t="str">
+        <v/>
+      </c>
+      <c r="K79" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2717,6 +3191,12 @@
         <v/>
       </c>
       <c r="I80" t="str">
+        <v/>
+      </c>
+      <c r="J80" t="str">
+        <v/>
+      </c>
+      <c r="K80" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2746,6 +3226,12 @@
         <v/>
       </c>
       <c r="I81" t="str">
+        <v/>
+      </c>
+      <c r="J81" t="str">
+        <v/>
+      </c>
+      <c r="K81" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2775,6 +3261,12 @@
         <v/>
       </c>
       <c r="I82" t="str">
+        <v/>
+      </c>
+      <c r="J82" t="str">
+        <v/>
+      </c>
+      <c r="K82" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2804,6 +3296,12 @@
         <v/>
       </c>
       <c r="I83" t="str">
+        <v/>
+      </c>
+      <c r="J83" t="str">
+        <v/>
+      </c>
+      <c r="K83" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2833,6 +3331,12 @@
         <v/>
       </c>
       <c r="I84" t="str">
+        <v/>
+      </c>
+      <c r="J84" t="str">
+        <v/>
+      </c>
+      <c r="K84" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2862,6 +3366,12 @@
         <v/>
       </c>
       <c r="I85" t="str">
+        <v/>
+      </c>
+      <c r="J85" t="str">
+        <v/>
+      </c>
+      <c r="K85" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2891,6 +3401,12 @@
         <v/>
       </c>
       <c r="I86" t="str">
+        <v/>
+      </c>
+      <c r="J86" t="str">
+        <v/>
+      </c>
+      <c r="K86" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2920,6 +3436,12 @@
         <v/>
       </c>
       <c r="I87" t="str">
+        <v/>
+      </c>
+      <c r="J87" t="str">
+        <v/>
+      </c>
+      <c r="K87" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2949,6 +3471,12 @@
         <v/>
       </c>
       <c r="I88" t="str">
+        <v/>
+      </c>
+      <c r="J88" t="str">
+        <v/>
+      </c>
+      <c r="K88" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -2978,6 +3506,12 @@
         <v/>
       </c>
       <c r="I89" t="str">
+        <v/>
+      </c>
+      <c r="J89" t="str">
+        <v/>
+      </c>
+      <c r="K89" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3007,6 +3541,12 @@
         <v/>
       </c>
       <c r="I90" t="str">
+        <v/>
+      </c>
+      <c r="J90" t="str">
+        <v/>
+      </c>
+      <c r="K90" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3036,6 +3576,12 @@
         <v/>
       </c>
       <c r="I91" t="str">
+        <v/>
+      </c>
+      <c r="J91" t="str">
+        <v/>
+      </c>
+      <c r="K91" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3065,6 +3611,12 @@
         <v/>
       </c>
       <c r="I92" t="str">
+        <v/>
+      </c>
+      <c r="J92" t="str">
+        <v/>
+      </c>
+      <c r="K92" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3094,6 +3646,12 @@
         <v/>
       </c>
       <c r="I93" t="str">
+        <v/>
+      </c>
+      <c r="J93" t="str">
+        <v/>
+      </c>
+      <c r="K93" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3123,6 +3681,12 @@
         <v/>
       </c>
       <c r="I94" t="str">
+        <v/>
+      </c>
+      <c r="J94" t="str">
+        <v/>
+      </c>
+      <c r="K94" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3152,6 +3716,12 @@
         <v/>
       </c>
       <c r="I95" t="str">
+        <v/>
+      </c>
+      <c r="J95" t="str">
+        <v/>
+      </c>
+      <c r="K95" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3181,6 +3751,12 @@
         <v/>
       </c>
       <c r="I96" t="str">
+        <v/>
+      </c>
+      <c r="J96" t="str">
+        <v/>
+      </c>
+      <c r="K96" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3210,6 +3786,12 @@
         <v/>
       </c>
       <c r="I97" t="str">
+        <v/>
+      </c>
+      <c r="J97" t="str">
+        <v/>
+      </c>
+      <c r="K97" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3239,6 +3821,12 @@
         <v/>
       </c>
       <c r="I98" t="str">
+        <v/>
+      </c>
+      <c r="J98" t="str">
+        <v/>
+      </c>
+      <c r="K98" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3268,6 +3856,12 @@
         <v/>
       </c>
       <c r="I99" t="str">
+        <v/>
+      </c>
+      <c r="J99" t="str">
+        <v/>
+      </c>
+      <c r="K99" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3297,6 +3891,12 @@
         <v/>
       </c>
       <c r="I100" t="str">
+        <v/>
+      </c>
+      <c r="J100" t="str">
+        <v/>
+      </c>
+      <c r="K100" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3326,6 +3926,12 @@
         <v/>
       </c>
       <c r="I101" t="str">
+        <v/>
+      </c>
+      <c r="J101" t="str">
+        <v/>
+      </c>
+      <c r="K101" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3355,6 +3961,12 @@
         <v/>
       </c>
       <c r="I102" t="str">
+        <v/>
+      </c>
+      <c r="J102" t="str">
+        <v/>
+      </c>
+      <c r="K102" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3384,6 +3996,12 @@
         <v/>
       </c>
       <c r="I103" t="str">
+        <v/>
+      </c>
+      <c r="J103" t="str">
+        <v/>
+      </c>
+      <c r="K103" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3413,6 +4031,12 @@
         <v/>
       </c>
       <c r="I104" t="str">
+        <v/>
+      </c>
+      <c r="J104" t="str">
+        <v/>
+      </c>
+      <c r="K104" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3442,6 +4066,12 @@
         <v/>
       </c>
       <c r="I105" t="str">
+        <v/>
+      </c>
+      <c r="J105" t="str">
+        <v/>
+      </c>
+      <c r="K105" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3471,6 +4101,12 @@
         <v/>
       </c>
       <c r="I106" t="str">
+        <v/>
+      </c>
+      <c r="J106" t="str">
+        <v/>
+      </c>
+      <c r="K106" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3500,6 +4136,12 @@
         <v/>
       </c>
       <c r="I107" t="str">
+        <v/>
+      </c>
+      <c r="J107" t="str">
+        <v/>
+      </c>
+      <c r="K107" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3529,6 +4171,12 @@
         <v/>
       </c>
       <c r="I108" t="str">
+        <v/>
+      </c>
+      <c r="J108" t="str">
+        <v/>
+      </c>
+      <c r="K108" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3558,6 +4206,12 @@
         <v/>
       </c>
       <c r="I109" t="str">
+        <v/>
+      </c>
+      <c r="J109" t="str">
+        <v/>
+      </c>
+      <c r="K109" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3578,15 +4232,21 @@
         <v/>
       </c>
       <c r="F110" t="str">
-        <v/>
+        <v>KG</v>
       </c>
       <c r="G110" t="str">
-        <v/>
+        <v>Pizza Mania MES-01-12-001; Le Lapin MES-LL-01-09-001</v>
       </c>
       <c r="H110" t="str">
         <v/>
       </c>
       <c r="I110" t="str">
+        <v/>
+      </c>
+      <c r="J110" t="str">
+        <v/>
+      </c>
+      <c r="K110" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3616,6 +4276,12 @@
         <v/>
       </c>
       <c r="I111" t="str">
+        <v/>
+      </c>
+      <c r="J111" t="str">
+        <v/>
+      </c>
+      <c r="K111" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3645,6 +4311,12 @@
         <v/>
       </c>
       <c r="I112" t="str">
+        <v/>
+      </c>
+      <c r="J112" t="str">
+        <v/>
+      </c>
+      <c r="K112" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3674,6 +4346,12 @@
         <v/>
       </c>
       <c r="I113" t="str">
+        <v/>
+      </c>
+      <c r="J113" t="str">
+        <v/>
+      </c>
+      <c r="K113" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3703,6 +4381,12 @@
         <v/>
       </c>
       <c r="I114" t="str">
+        <v/>
+      </c>
+      <c r="J114" t="str">
+        <v/>
+      </c>
+      <c r="K114" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3732,6 +4416,12 @@
         <v/>
       </c>
       <c r="I115" t="str">
+        <v/>
+      </c>
+      <c r="J115" t="str">
+        <v/>
+      </c>
+      <c r="K115" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3761,6 +4451,12 @@
         <v/>
       </c>
       <c r="I116" t="str">
+        <v/>
+      </c>
+      <c r="J116" t="str">
+        <v/>
+      </c>
+      <c r="K116" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3790,6 +4486,12 @@
         <v/>
       </c>
       <c r="I117" t="str">
+        <v/>
+      </c>
+      <c r="J117" t="str">
+        <v/>
+      </c>
+      <c r="K117" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3819,6 +4521,12 @@
         <v/>
       </c>
       <c r="I118" t="str">
+        <v/>
+      </c>
+      <c r="J118" t="str">
+        <v/>
+      </c>
+      <c r="K118" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3848,6 +4556,12 @@
         <v/>
       </c>
       <c r="I119" t="str">
+        <v/>
+      </c>
+      <c r="J119" t="str">
+        <v/>
+      </c>
+      <c r="K119" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3877,6 +4591,12 @@
         <v/>
       </c>
       <c r="I120" t="str">
+        <v/>
+      </c>
+      <c r="J120" t="str">
+        <v/>
+      </c>
+      <c r="K120" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3906,6 +4626,12 @@
         <v/>
       </c>
       <c r="I121" t="str">
+        <v/>
+      </c>
+      <c r="J121" t="str">
+        <v/>
+      </c>
+      <c r="K121" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3935,6 +4661,12 @@
         <v/>
       </c>
       <c r="I122" t="str">
+        <v/>
+      </c>
+      <c r="J122" t="str">
+        <v/>
+      </c>
+      <c r="K122" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3964,6 +4696,12 @@
         <v/>
       </c>
       <c r="I123" t="str">
+        <v/>
+      </c>
+      <c r="J123" t="str">
+        <v/>
+      </c>
+      <c r="K123" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -3993,6 +4731,12 @@
         <v/>
       </c>
       <c r="I124" t="str">
+        <v/>
+      </c>
+      <c r="J124" t="str">
+        <v/>
+      </c>
+      <c r="K124" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4022,6 +4766,12 @@
         <v/>
       </c>
       <c r="I125" t="str">
+        <v/>
+      </c>
+      <c r="J125" t="str">
+        <v/>
+      </c>
+      <c r="K125" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4042,15 +4792,21 @@
         <v/>
       </c>
       <c r="F126" t="str">
-        <v/>
+        <v>KG</v>
       </c>
       <c r="G126" t="str">
-        <v/>
+        <v>Pizza Mania CHS-01-01-010</v>
       </c>
       <c r="H126" t="str">
         <v/>
       </c>
       <c r="I126" t="str">
+        <v/>
+      </c>
+      <c r="J126" t="str">
+        <v/>
+      </c>
+      <c r="K126" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4080,6 +4836,12 @@
         <v/>
       </c>
       <c r="I127" t="str">
+        <v/>
+      </c>
+      <c r="J127" t="str">
+        <v/>
+      </c>
+      <c r="K127" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4109,6 +4871,12 @@
         <v/>
       </c>
       <c r="I128" t="str">
+        <v/>
+      </c>
+      <c r="J128" t="str">
+        <v/>
+      </c>
+      <c r="K128" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4138,6 +4906,12 @@
         <v/>
       </c>
       <c r="I129" t="str">
+        <v/>
+      </c>
+      <c r="J129" t="str">
+        <v/>
+      </c>
+      <c r="K129" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4167,6 +4941,12 @@
         <v/>
       </c>
       <c r="I130" t="str">
+        <v/>
+      </c>
+      <c r="J130" t="str">
+        <v/>
+      </c>
+      <c r="K130" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4196,6 +4976,12 @@
         <v/>
       </c>
       <c r="I131" t="str">
+        <v/>
+      </c>
+      <c r="J131" t="str">
+        <v/>
+      </c>
+      <c r="K131" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4225,6 +5011,12 @@
         <v/>
       </c>
       <c r="I132" t="str">
+        <v/>
+      </c>
+      <c r="J132" t="str">
+        <v/>
+      </c>
+      <c r="K132" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4254,6 +5046,12 @@
         <v/>
       </c>
       <c r="I133" t="str">
+        <v/>
+      </c>
+      <c r="J133" t="str">
+        <v/>
+      </c>
+      <c r="K133" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4283,6 +5081,12 @@
         <v/>
       </c>
       <c r="I134" t="str">
+        <v/>
+      </c>
+      <c r="J134" t="str">
+        <v/>
+      </c>
+      <c r="K134" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4312,6 +5116,12 @@
         <v/>
       </c>
       <c r="I135" t="str">
+        <v/>
+      </c>
+      <c r="J135" t="str">
+        <v/>
+      </c>
+      <c r="K135" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4341,6 +5151,12 @@
         <v/>
       </c>
       <c r="I136" t="str">
+        <v/>
+      </c>
+      <c r="J136" t="str">
+        <v/>
+      </c>
+      <c r="K136" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4370,6 +5186,12 @@
         <v/>
       </c>
       <c r="I137" t="str">
+        <v/>
+      </c>
+      <c r="J137" t="str">
+        <v/>
+      </c>
+      <c r="K137" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4399,6 +5221,12 @@
         <v/>
       </c>
       <c r="I138" t="str">
+        <v/>
+      </c>
+      <c r="J138" t="str">
+        <v/>
+      </c>
+      <c r="K138" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4428,6 +5256,12 @@
         <v/>
       </c>
       <c r="I139" t="str">
+        <v/>
+      </c>
+      <c r="J139" t="str">
+        <v/>
+      </c>
+      <c r="K139" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4457,6 +5291,12 @@
         <v/>
       </c>
       <c r="I140" t="str">
+        <v/>
+      </c>
+      <c r="J140" t="str">
+        <v/>
+      </c>
+      <c r="K140" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4486,6 +5326,12 @@
         <v/>
       </c>
       <c r="I141" t="str">
+        <v/>
+      </c>
+      <c r="J141" t="str">
+        <v/>
+      </c>
+      <c r="K141" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4515,6 +5361,12 @@
         <v/>
       </c>
       <c r="I142" t="str">
+        <v/>
+      </c>
+      <c r="J142" t="str">
+        <v/>
+      </c>
+      <c r="K142" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4544,6 +5396,12 @@
         <v/>
       </c>
       <c r="I143" t="str">
+        <v/>
+      </c>
+      <c r="J143" t="str">
+        <v/>
+      </c>
+      <c r="K143" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4573,6 +5431,12 @@
         <v/>
       </c>
       <c r="I144" t="str">
+        <v/>
+      </c>
+      <c r="J144" t="str">
+        <v/>
+      </c>
+      <c r="K144" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4602,6 +5466,12 @@
         <v/>
       </c>
       <c r="I145" t="str">
+        <v/>
+      </c>
+      <c r="J145" t="str">
+        <v/>
+      </c>
+      <c r="K145" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4631,6 +5501,12 @@
         <v/>
       </c>
       <c r="I146" t="str">
+        <v/>
+      </c>
+      <c r="J146" t="str">
+        <v/>
+      </c>
+      <c r="K146" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4660,6 +5536,12 @@
         <v/>
       </c>
       <c r="I147" t="str">
+        <v/>
+      </c>
+      <c r="J147" t="str">
+        <v/>
+      </c>
+      <c r="K147" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4689,6 +5571,12 @@
         <v/>
       </c>
       <c r="I148" t="str">
+        <v/>
+      </c>
+      <c r="J148" t="str">
+        <v/>
+      </c>
+      <c r="K148" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4718,6 +5606,12 @@
         <v/>
       </c>
       <c r="I149" t="str">
+        <v/>
+      </c>
+      <c r="J149" t="str">
+        <v/>
+      </c>
+      <c r="K149" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4747,6 +5641,12 @@
         <v/>
       </c>
       <c r="I150" t="str">
+        <v/>
+      </c>
+      <c r="J150" t="str">
+        <v/>
+      </c>
+      <c r="K150" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4776,6 +5676,12 @@
         <v/>
       </c>
       <c r="I151" t="str">
+        <v/>
+      </c>
+      <c r="J151" t="str">
+        <v/>
+      </c>
+      <c r="K151" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4805,6 +5711,12 @@
         <v/>
       </c>
       <c r="I152" t="str">
+        <v/>
+      </c>
+      <c r="J152" t="str">
+        <v/>
+      </c>
+      <c r="K152" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4834,6 +5746,12 @@
         <v/>
       </c>
       <c r="I153" t="str">
+        <v/>
+      </c>
+      <c r="J153" t="str">
+        <v/>
+      </c>
+      <c r="K153" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4863,6 +5781,12 @@
         <v/>
       </c>
       <c r="I154" t="str">
+        <v/>
+      </c>
+      <c r="J154" t="str">
+        <v/>
+      </c>
+      <c r="K154" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4892,6 +5816,12 @@
         <v/>
       </c>
       <c r="I155" t="str">
+        <v/>
+      </c>
+      <c r="J155" t="str">
+        <v/>
+      </c>
+      <c r="K155" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4921,6 +5851,12 @@
         <v/>
       </c>
       <c r="I156" t="str">
+        <v/>
+      </c>
+      <c r="J156" t="str">
+        <v/>
+      </c>
+      <c r="K156" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4950,6 +5886,12 @@
         <v/>
       </c>
       <c r="I157" t="str">
+        <v/>
+      </c>
+      <c r="J157" t="str">
+        <v/>
+      </c>
+      <c r="K157" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -4979,6 +5921,12 @@
         <v/>
       </c>
       <c r="I158" t="str">
+        <v/>
+      </c>
+      <c r="J158" t="str">
+        <v/>
+      </c>
+      <c r="K158" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5008,6 +5956,12 @@
         <v/>
       </c>
       <c r="I159" t="str">
+        <v/>
+      </c>
+      <c r="J159" t="str">
+        <v/>
+      </c>
+      <c r="K159" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5037,6 +5991,12 @@
         <v/>
       </c>
       <c r="I160" t="str">
+        <v/>
+      </c>
+      <c r="J160" t="str">
+        <v/>
+      </c>
+      <c r="K160" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5066,6 +6026,12 @@
         <v/>
       </c>
       <c r="I161" t="str">
+        <v/>
+      </c>
+      <c r="J161" t="str">
+        <v/>
+      </c>
+      <c r="K161" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5095,6 +6061,12 @@
         <v/>
       </c>
       <c r="I162" t="str">
+        <v/>
+      </c>
+      <c r="J162" t="str">
+        <v/>
+      </c>
+      <c r="K162" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5124,6 +6096,12 @@
         <v/>
       </c>
       <c r="I163" t="str">
+        <v/>
+      </c>
+      <c r="J163" t="str">
+        <v/>
+      </c>
+      <c r="K163" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5153,6 +6131,12 @@
         <v/>
       </c>
       <c r="I164" t="str">
+        <v/>
+      </c>
+      <c r="J164" t="str">
+        <v/>
+      </c>
+      <c r="K164" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5182,6 +6166,12 @@
         <v/>
       </c>
       <c r="I165" t="str">
+        <v/>
+      </c>
+      <c r="J165" t="str">
+        <v/>
+      </c>
+      <c r="K165" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5211,6 +6201,12 @@
         <v/>
       </c>
       <c r="I166" t="str">
+        <v/>
+      </c>
+      <c r="J166" t="str">
+        <v/>
+      </c>
+      <c r="K166" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5240,6 +6236,12 @@
         <v/>
       </c>
       <c r="I167" t="str">
+        <v/>
+      </c>
+      <c r="J167" t="str">
+        <v/>
+      </c>
+      <c r="K167" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5269,6 +6271,12 @@
         <v/>
       </c>
       <c r="I168" t="str">
+        <v/>
+      </c>
+      <c r="J168" t="str">
+        <v/>
+      </c>
+      <c r="K168" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5289,15 +6297,21 @@
         <v/>
       </c>
       <c r="F169" t="str">
-        <v/>
+        <v>EA</v>
       </c>
       <c r="G169" t="str">
-        <v/>
+        <v>Pizza Mania SEAS-01-06-002; Le Lapin SEAS-LL-01-11-001; Le Lapin SEAS-LL-01-11-002; Le Lapin SEAS-LL-01-11-003</v>
       </c>
       <c r="H169" t="str">
         <v/>
       </c>
       <c r="I169" t="str">
+        <v/>
+      </c>
+      <c r="J169" t="str">
+        <v/>
+      </c>
+      <c r="K169" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5327,6 +6341,12 @@
         <v/>
       </c>
       <c r="I170" t="str">
+        <v/>
+      </c>
+      <c r="J170" t="str">
+        <v/>
+      </c>
+      <c r="K170" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5356,6 +6376,12 @@
         <v/>
       </c>
       <c r="I171" t="str">
+        <v/>
+      </c>
+      <c r="J171" t="str">
+        <v/>
+      </c>
+      <c r="K171" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5385,6 +6411,12 @@
         <v/>
       </c>
       <c r="I172" t="str">
+        <v/>
+      </c>
+      <c r="J172" t="str">
+        <v/>
+      </c>
+      <c r="K172" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5414,6 +6446,12 @@
         <v/>
       </c>
       <c r="I173" t="str">
+        <v/>
+      </c>
+      <c r="J173" t="str">
+        <v/>
+      </c>
+      <c r="K173" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5443,6 +6481,12 @@
         <v/>
       </c>
       <c r="I174" t="str">
+        <v/>
+      </c>
+      <c r="J174" t="str">
+        <v/>
+      </c>
+      <c r="K174" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5472,6 +6516,12 @@
         <v/>
       </c>
       <c r="I175" t="str">
+        <v/>
+      </c>
+      <c r="J175" t="str">
+        <v/>
+      </c>
+      <c r="K175" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5501,6 +6551,12 @@
         <v/>
       </c>
       <c r="I176" t="str">
+        <v/>
+      </c>
+      <c r="J176" t="str">
+        <v/>
+      </c>
+      <c r="K176" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5530,6 +6586,12 @@
         <v/>
       </c>
       <c r="I177" t="str">
+        <v/>
+      </c>
+      <c r="J177" t="str">
+        <v/>
+      </c>
+      <c r="K177" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5559,6 +6621,12 @@
         <v/>
       </c>
       <c r="I178" t="str">
+        <v/>
+      </c>
+      <c r="J178" t="str">
+        <v/>
+      </c>
+      <c r="K178" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5588,6 +6656,12 @@
         <v/>
       </c>
       <c r="I179" t="str">
+        <v/>
+      </c>
+      <c r="J179" t="str">
+        <v/>
+      </c>
+      <c r="K179" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5617,6 +6691,12 @@
         <v/>
       </c>
       <c r="I180" t="str">
+        <v/>
+      </c>
+      <c r="J180" t="str">
+        <v/>
+      </c>
+      <c r="K180" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5646,6 +6726,12 @@
         <v/>
       </c>
       <c r="I181" t="str">
+        <v/>
+      </c>
+      <c r="J181" t="str">
+        <v/>
+      </c>
+      <c r="K181" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5675,6 +6761,12 @@
         <v/>
       </c>
       <c r="I182" t="str">
+        <v/>
+      </c>
+      <c r="J182" t="str">
+        <v/>
+      </c>
+      <c r="K182" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5704,6 +6796,12 @@
         <v/>
       </c>
       <c r="I183" t="str">
+        <v/>
+      </c>
+      <c r="J183" t="str">
+        <v/>
+      </c>
+      <c r="K183" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5733,6 +6831,12 @@
         <v/>
       </c>
       <c r="I184" t="str">
+        <v/>
+      </c>
+      <c r="J184" t="str">
+        <v/>
+      </c>
+      <c r="K184" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5762,6 +6866,12 @@
         <v/>
       </c>
       <c r="I185" t="str">
+        <v/>
+      </c>
+      <c r="J185" t="str">
+        <v/>
+      </c>
+      <c r="K185" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5791,6 +6901,12 @@
         <v/>
       </c>
       <c r="I186" t="str">
+        <v/>
+      </c>
+      <c r="J186" t="str">
+        <v/>
+      </c>
+      <c r="K186" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5820,6 +6936,12 @@
         <v/>
       </c>
       <c r="I187" t="str">
+        <v/>
+      </c>
+      <c r="J187" t="str">
+        <v/>
+      </c>
+      <c r="K187" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5849,6 +6971,12 @@
         <v/>
       </c>
       <c r="I188" t="str">
+        <v/>
+      </c>
+      <c r="J188" t="str">
+        <v/>
+      </c>
+      <c r="K188" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5878,6 +7006,12 @@
         <v/>
       </c>
       <c r="I189" t="str">
+        <v/>
+      </c>
+      <c r="J189" t="str">
+        <v/>
+      </c>
+      <c r="K189" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5907,6 +7041,12 @@
         <v/>
       </c>
       <c r="I190" t="str">
+        <v/>
+      </c>
+      <c r="J190" t="str">
+        <v/>
+      </c>
+      <c r="K190" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5936,6 +7076,12 @@
         <v/>
       </c>
       <c r="I191" t="str">
+        <v/>
+      </c>
+      <c r="J191" t="str">
+        <v/>
+      </c>
+      <c r="K191" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5965,6 +7111,12 @@
         <v/>
       </c>
       <c r="I192" t="str">
+        <v/>
+      </c>
+      <c r="J192" t="str">
+        <v/>
+      </c>
+      <c r="K192" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -5994,6 +7146,12 @@
         <v/>
       </c>
       <c r="I193" t="str">
+        <v/>
+      </c>
+      <c r="J193" t="str">
+        <v/>
+      </c>
+      <c r="K193" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6023,6 +7181,12 @@
         <v/>
       </c>
       <c r="I194" t="str">
+        <v/>
+      </c>
+      <c r="J194" t="str">
+        <v/>
+      </c>
+      <c r="K194" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6052,6 +7216,12 @@
         <v/>
       </c>
       <c r="I195" t="str">
+        <v/>
+      </c>
+      <c r="J195" t="str">
+        <v/>
+      </c>
+      <c r="K195" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6081,6 +7251,12 @@
         <v/>
       </c>
       <c r="I196" t="str">
+        <v/>
+      </c>
+      <c r="J196" t="str">
+        <v/>
+      </c>
+      <c r="K196" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6110,6 +7286,12 @@
         <v/>
       </c>
       <c r="I197" t="str">
+        <v/>
+      </c>
+      <c r="J197" t="str">
+        <v/>
+      </c>
+      <c r="K197" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6139,6 +7321,12 @@
         <v/>
       </c>
       <c r="I198" t="str">
+        <v/>
+      </c>
+      <c r="J198" t="str">
+        <v/>
+      </c>
+      <c r="K198" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6168,6 +7356,12 @@
         <v/>
       </c>
       <c r="I199" t="str">
+        <v/>
+      </c>
+      <c r="J199" t="str">
+        <v/>
+      </c>
+      <c r="K199" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6197,6 +7391,12 @@
         <v/>
       </c>
       <c r="I200" t="str">
+        <v/>
+      </c>
+      <c r="J200" t="str">
+        <v/>
+      </c>
+      <c r="K200" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6226,6 +7426,12 @@
         <v/>
       </c>
       <c r="I201" t="str">
+        <v/>
+      </c>
+      <c r="J201" t="str">
+        <v/>
+      </c>
+      <c r="K201" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6255,6 +7461,12 @@
         <v/>
       </c>
       <c r="I202" t="str">
+        <v/>
+      </c>
+      <c r="J202" t="str">
+        <v/>
+      </c>
+      <c r="K202" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6284,6 +7496,12 @@
         <v/>
       </c>
       <c r="I203" t="str">
+        <v/>
+      </c>
+      <c r="J203" t="str">
+        <v/>
+      </c>
+      <c r="K203" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6313,6 +7531,12 @@
         <v/>
       </c>
       <c r="I204" t="str">
+        <v/>
+      </c>
+      <c r="J204" t="str">
+        <v/>
+      </c>
+      <c r="K204" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6342,6 +7566,12 @@
         <v/>
       </c>
       <c r="I205" t="str">
+        <v/>
+      </c>
+      <c r="J205" t="str">
+        <v/>
+      </c>
+      <c r="K205" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6371,6 +7601,12 @@
         <v/>
       </c>
       <c r="I206" t="str">
+        <v/>
+      </c>
+      <c r="J206" t="str">
+        <v/>
+      </c>
+      <c r="K206" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6400,6 +7636,12 @@
         <v/>
       </c>
       <c r="I207" t="str">
+        <v/>
+      </c>
+      <c r="J207" t="str">
+        <v/>
+      </c>
+      <c r="K207" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6429,6 +7671,12 @@
         <v/>
       </c>
       <c r="I208" t="str">
+        <v/>
+      </c>
+      <c r="J208" t="str">
+        <v/>
+      </c>
+      <c r="K208" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6458,6 +7706,12 @@
         <v/>
       </c>
       <c r="I209" t="str">
+        <v/>
+      </c>
+      <c r="J209" t="str">
+        <v/>
+      </c>
+      <c r="K209" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6487,6 +7741,12 @@
         <v/>
       </c>
       <c r="I210" t="str">
+        <v/>
+      </c>
+      <c r="J210" t="str">
+        <v/>
+      </c>
+      <c r="K210" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6516,6 +7776,12 @@
         <v/>
       </c>
       <c r="I211" t="str">
+        <v/>
+      </c>
+      <c r="J211" t="str">
+        <v/>
+      </c>
+      <c r="K211" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6545,6 +7811,12 @@
         <v/>
       </c>
       <c r="I212" t="str">
+        <v/>
+      </c>
+      <c r="J212" t="str">
+        <v/>
+      </c>
+      <c r="K212" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6574,6 +7846,12 @@
         <v/>
       </c>
       <c r="I213" t="str">
+        <v/>
+      </c>
+      <c r="J213" t="str">
+        <v/>
+      </c>
+      <c r="K213" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6603,6 +7881,12 @@
         <v/>
       </c>
       <c r="I214" t="str">
+        <v/>
+      </c>
+      <c r="J214" t="str">
+        <v/>
+      </c>
+      <c r="K214" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6632,6 +7916,12 @@
         <v/>
       </c>
       <c r="I215" t="str">
+        <v/>
+      </c>
+      <c r="J215" t="str">
+        <v/>
+      </c>
+      <c r="K215" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6661,6 +7951,12 @@
         <v/>
       </c>
       <c r="I216" t="str">
+        <v/>
+      </c>
+      <c r="J216" t="str">
+        <v/>
+      </c>
+      <c r="K216" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6690,6 +7986,12 @@
         <v/>
       </c>
       <c r="I217" t="str">
+        <v/>
+      </c>
+      <c r="J217" t="str">
+        <v/>
+      </c>
+      <c r="K217" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6719,6 +8021,12 @@
         <v/>
       </c>
       <c r="I218" t="str">
+        <v/>
+      </c>
+      <c r="J218" t="str">
+        <v/>
+      </c>
+      <c r="K218" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6748,6 +8056,12 @@
         <v/>
       </c>
       <c r="I219" t="str">
+        <v/>
+      </c>
+      <c r="J219" t="str">
+        <v/>
+      </c>
+      <c r="K219" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6777,6 +8091,12 @@
         <v/>
       </c>
       <c r="I220" t="str">
+        <v/>
+      </c>
+      <c r="J220" t="str">
+        <v/>
+      </c>
+      <c r="K220" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6806,6 +8126,12 @@
         <v/>
       </c>
       <c r="I221" t="str">
+        <v/>
+      </c>
+      <c r="J221" t="str">
+        <v/>
+      </c>
+      <c r="K221" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6835,6 +8161,12 @@
         <v/>
       </c>
       <c r="I222" t="str">
+        <v/>
+      </c>
+      <c r="J222" t="str">
+        <v/>
+      </c>
+      <c r="K222" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6864,6 +8196,12 @@
         <v/>
       </c>
       <c r="I223" t="str">
+        <v/>
+      </c>
+      <c r="J223" t="str">
+        <v/>
+      </c>
+      <c r="K223" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6893,6 +8231,12 @@
         <v/>
       </c>
       <c r="I224" t="str">
+        <v/>
+      </c>
+      <c r="J224" t="str">
+        <v/>
+      </c>
+      <c r="K224" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6922,6 +8266,12 @@
         <v/>
       </c>
       <c r="I225" t="str">
+        <v/>
+      </c>
+      <c r="J225" t="str">
+        <v/>
+      </c>
+      <c r="K225" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6951,6 +8301,12 @@
         <v/>
       </c>
       <c r="I226" t="str">
+        <v/>
+      </c>
+      <c r="J226" t="str">
+        <v/>
+      </c>
+      <c r="K226" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -6980,6 +8336,12 @@
         <v/>
       </c>
       <c r="I227" t="str">
+        <v/>
+      </c>
+      <c r="J227" t="str">
+        <v/>
+      </c>
+      <c r="K227" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -7009,6 +8371,12 @@
         <v/>
       </c>
       <c r="I228" t="str">
+        <v/>
+      </c>
+      <c r="J228" t="str">
+        <v/>
+      </c>
+      <c r="K228" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
@@ -7038,19 +8406,25 @@
         <v/>
       </c>
       <c r="I229" t="str">
+        <v/>
+      </c>
+      <c r="J229" t="str">
+        <v/>
+      </c>
+      <c r="K229" t="str">
         <v>MISSING_UNIT</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:I229"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K229"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -7059,47 +8433,63 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>proposedUnit</v>
+        <v>Allowed units</v>
       </c>
       <c r="B2" t="str">
-        <v>the unit it is bought and counted in, e.g. KG, EA, Pack, Bottle</v>
+        <v>KG, EA, Pack, Carton — the same as Pizza Mania and Le Lapin, with Carton instead of Bottle</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>baseUnit</v>
+        <v>suggestedUnit</v>
       </c>
       <c r="B3" t="str">
-        <v>the stock unit; blank = same as proposedUnit</v>
+        <v>the unit the SAME product has in Pizza Mania / Le Lapin (suggestedFrom says which). Copy it to proposedUnit only if it is right; it is never applied by itself</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>conversionFactor</v>
+        <v>proposedUnit</v>
       </c>
       <c r="B4" t="str">
-        <v>how many baseUnit in ONE proposedUnit (e.g. 1 Pack = 12 EA → 12); only when the units differ</v>
+        <v>the unit it is bought and counted in</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>supplierId</v>
+        <v>baseUnit</v>
       </c>
       <c r="B5" t="str">
-        <v>left blank: suppliers are linked in the app, never guessed from the name</v>
+        <v>the stock unit; blank = same as proposedUnit</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>conversionFactor</v>
+      </c>
+      <c r="B6" t="str">
+        <v>how many baseUnit in ONE proposedUnit (e.g. 1 Carton = 12 EA → 12); only when the units differ</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>supplierId</v>
+      </c>
+      <c r="B7" t="str">
+        <v>left blank: suppliers are linked in the app, never guessed from the name</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
         <v>Check before applying</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B8" t="str">
         <v>node scripts/rnd-units.mjs validate &lt;this file&gt;  (dry run, writes nothing)</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>